<commit_message>
made changes to calculations
</commit_message>
<xml_diff>
--- a/cfm_journal/data/Juice_Ledger_Christie.xlsx
+++ b/cfm_journal/data/Juice_Ledger_Christie.xlsx
@@ -11,7 +11,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -41,8 +43,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -445,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L125"/>
+  <dimension ref="A1:L132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8048,6 +8051,356 @@
         </is>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B126" s="1" t="n">
+        <v>46014.53680555556</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>2</v>
+      </c>
+      <c r="F126" t="n">
+        <v>134</v>
+      </c>
+      <c r="G126" s="1" t="n">
+        <v>46024</v>
+      </c>
+      <c r="H126" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="I126" t="n">
+        <v>136.6375</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>ABNB|134.0|2026-01-02|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B127" s="1" t="n">
+        <v>46021.43819444445</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>2</v>
+      </c>
+      <c r="F127" t="n">
+        <v>134</v>
+      </c>
+      <c r="G127" s="1" t="n">
+        <v>46024</v>
+      </c>
+      <c r="H127" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="I127" t="n">
+        <v>137.3563</v>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>ABNB|134.0|2026-01-02|CALL|CLOSE</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B128" s="1" t="n">
+        <v>46021.49930555555</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>2</v>
+      </c>
+      <c r="F128" t="n">
+        <v>135</v>
+      </c>
+      <c r="G128" s="1" t="n">
+        <v>46031</v>
+      </c>
+      <c r="H128" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="I128" t="n">
+        <v>137.035</v>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>ABNB|135.0|2026-01-09|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B129" s="1" t="n">
+        <v>46024.3625</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>2</v>
+      </c>
+      <c r="F129" t="n">
+        <v>135</v>
+      </c>
+      <c r="G129" s="1" t="n">
+        <v>46031</v>
+      </c>
+      <c r="H129" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="I129" t="n">
+        <v>133.825</v>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>ABNB|135.0|2026-01-09|CALL|CLOSE</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B130" s="1" t="n">
+        <v>46024.3625</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>2</v>
+      </c>
+      <c r="F130" t="n">
+        <v>132</v>
+      </c>
+      <c r="G130" s="1" t="n">
+        <v>46031</v>
+      </c>
+      <c r="H130" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="I130" t="n">
+        <v>133.825</v>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>ABNB|132.0|2026-01-09|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B131" s="1" t="n">
+        <v>46027.47152777778</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>2</v>
+      </c>
+      <c r="F131" t="n">
+        <v>132</v>
+      </c>
+      <c r="G131" s="1" t="n">
+        <v>46031</v>
+      </c>
+      <c r="H131" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="I131" t="n">
+        <v>137.53</v>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>ABNB|132.0|2026-01-09|CALL|CLOSE</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B132" s="1" t="n">
+        <v>46027.47152777778</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>2</v>
+      </c>
+      <c r="F132" t="n">
+        <v>134</v>
+      </c>
+      <c r="G132" s="1" t="n">
+        <v>46031</v>
+      </c>
+      <c r="H132" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="I132" t="n">
+        <v>137.53</v>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>ABNB|134.0|2026-01-09|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
adding changes for dashboard calculations
</commit_message>
<xml_diff>
--- a/cfm_journal/data/Juice_Ledger_Christie.xlsx
+++ b/cfm_journal/data/Juice_Ledger_Christie.xlsx
@@ -1,11 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
-    <sheet name="Ledger" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -14,7 +18,14 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -23,12 +34,15 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill/>
     </fill>
   </fills>
   <borders count="1">
@@ -41,16 +55,16 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -449,7 +463,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M109"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="0"/>
+  <cols>
+    <col width="17.875" customWidth="1" min="2" max="2"/>
+    <col width="16.75" customWidth="1" min="7" max="7"/>
+    <col width="32.75" customWidth="1" min="10" max="10"/>
+    <col width="33.25" customWidth="1" min="12" max="12"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -6084,7 +6104,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>cb86935f-1733-40f0-8ad6-fefb17700dd5</t>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
         </is>
       </c>
     </row>
@@ -6352,7 +6372,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>cb86935f-1733-40f0-8ad6-fefb17700dd5</t>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
         </is>
       </c>
     </row>
@@ -6419,7 +6439,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>cb86935f-1733-40f0-8ad6-fefb17700dd6</t>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
         </is>
       </c>
     </row>
@@ -6486,7 +6506,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>cb86935f-1733-40f0-8ad6-fefb17700dd7</t>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
         </is>
       </c>
     </row>
@@ -6620,7 +6640,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>cb86935f-1733-40f0-8ad6-fefb17700dd5</t>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6707,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>cb86935f-1733-40f0-8ad6-fefb17700dd4</t>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
         </is>
       </c>
     </row>
@@ -6821,7 +6841,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>cb86935f-1733-40f0-8ad6-fefb17700dd2</t>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
         </is>
       </c>
     </row>
@@ -6888,7 +6908,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>cb86935f-1733-40f0-8ad6-fefb17700dd1</t>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
         </is>
       </c>
     </row>
@@ -6955,7 +6975,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>cb86935f-1733-40f0-8ad6-fefb17700dd0</t>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
         </is>
       </c>
     </row>
@@ -7022,7 +7042,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>cb86935f-1733-40f0-8ad6-fefb17700dd1</t>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
         </is>
       </c>
     </row>
@@ -7089,7 +7109,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>cb86935f-1733-40f0-8ad6-fefb17700dd2</t>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
         </is>
       </c>
     </row>
@@ -7527,7 +7547,7 @@
         <v>9.199999999999999</v>
       </c>
       <c r="I108" t="n">
-        <v>184.9626</v>
+        <v>188.5525</v>
       </c>
       <c r="J108" t="inlineStr">
         <is>
@@ -7582,7 +7602,7 @@
         <v>8.800000000000001</v>
       </c>
       <c r="I109" t="n">
-        <v>184.9626</v>
+        <v>188.4175</v>
       </c>
       <c r="J109" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
pushing new calc changes
</commit_message>
<xml_diff>
--- a/cfm_journal/data/Juice_Ledger_Christie.xlsx
+++ b/cfm_journal/data/Juice_Ledger_Christie.xlsx
@@ -3,20 +3,21 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-23148" yWindow="4188" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="171027" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -57,9 +58,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -462,13 +465,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M109"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="0"/>
+  <dimension ref="A1:M124"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col width="17.875" customWidth="1" min="2" max="2"/>
-    <col width="16.75" customWidth="1" min="7" max="7"/>
-    <col width="32.75" customWidth="1" min="10" max="10"/>
-    <col width="33.25" customWidth="1" min="12" max="12"/>
+    <col width="20.42578125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="19.28515625" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="32.7109375" customWidth="1" min="10" max="10"/>
+    <col width="33.28515625" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7377,7 +7380,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>82f856ad-3a84-40d1-884d-02cc88c35c8a</t>
+          <t>c424d059-5cb0-43ea-8326-c6d950c300e0</t>
         </is>
       </c>
     </row>
@@ -7622,6 +7625,831 @@
       <c r="M109" t="inlineStr">
         <is>
           <t>82f856ad-3a84-40d1-884d-02cc88c35c8a</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="n">
+        <v>46029.38194444445</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>2</v>
+      </c>
+      <c r="F110" t="n">
+        <v>181</v>
+      </c>
+      <c r="G110" s="2" t="n">
+        <v>46038</v>
+      </c>
+      <c r="H110" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="I110" t="n">
+        <v>190.6575</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>NVDA|181.0|2026-01-16|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>82f856ad-3a84-40d1-884d-02cc88c35c8a</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="n">
+        <v>46036.39583333334</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>2</v>
+      </c>
+      <c r="F111" t="n">
+        <v>181</v>
+      </c>
+      <c r="G111" s="2" t="n">
+        <v>46038</v>
+      </c>
+      <c r="H111" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="I111" t="n">
+        <v>181.7037</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>NVDA|181.0|2026-01-16|CALL|CLOSE</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>82f856ad-3a84-40d1-884d-02cc88c35c8a</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="n">
+        <v>46036.39583333334</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>1</v>
+      </c>
+      <c r="F112" t="n">
+        <v>181</v>
+      </c>
+      <c r="G112" s="3" t="n">
+        <v>46038</v>
+      </c>
+      <c r="H112" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="I112" t="n">
+        <v>181.7037</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>NVDA|181.0|2026-01-16|CALL|CLOSE</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>c424d059-5cb0-43ea-8326-c6d950c300e0</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="n">
+        <v>46036.39583333334</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>1</v>
+      </c>
+      <c r="F113" t="n">
+        <v>179</v>
+      </c>
+      <c r="G113" s="3" t="n">
+        <v>46038</v>
+      </c>
+      <c r="H113" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="I113" t="n">
+        <v>181.7037</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>NVDA|179.0|2026-01-16|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>c424d059-5cb0-43ea-8326-c6d950c300e0</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="n">
+        <v>46036.39583333334</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>2</v>
+      </c>
+      <c r="F114" t="n">
+        <v>179</v>
+      </c>
+      <c r="G114" s="3" t="n">
+        <v>46038</v>
+      </c>
+      <c r="H114" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="I114" t="n">
+        <v>181.7037</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>NVDA|179.0|2026-01-16|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>82f856ad-3a84-40d1-884d-02cc88c35c8a</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B115" s="3" t="n">
+        <v>46037.37152777778</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>1</v>
+      </c>
+      <c r="F115" t="n">
+        <v>179</v>
+      </c>
+      <c r="G115" s="3" t="n">
+        <v>46038</v>
+      </c>
+      <c r="H115" t="n">
+        <v>9.59</v>
+      </c>
+      <c r="I115" t="n">
+        <v>188.3986</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>NVDA|179.0|2026-01-16|CALL|CLOSE</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>c424d059-5cb0-43ea-8326-c6d950c300e0</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="n">
+        <v>46037.37152777778</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>2</v>
+      </c>
+      <c r="F116" t="n">
+        <v>179</v>
+      </c>
+      <c r="G116" s="3" t="n">
+        <v>46038</v>
+      </c>
+      <c r="H116" t="n">
+        <v>9.59</v>
+      </c>
+      <c r="I116" t="n">
+        <v>188.3986</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>NVDA|179.0|2026-01-16|CALL|CLOSE</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>82f856ad-3a84-40d1-884d-02cc88c35c8a</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B117" s="3" t="n">
+        <v>46037.37152777778</v>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>2</v>
+      </c>
+      <c r="F117" t="n">
+        <v>180</v>
+      </c>
+      <c r="G117" s="3" t="n">
+        <v>46045</v>
+      </c>
+      <c r="H117" t="n">
+        <v>9.49</v>
+      </c>
+      <c r="I117" t="n">
+        <v>188.3986</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>NVDA|180.0|2026-01-23|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>82f856ad-3a84-40d1-884d-02cc88c35c8a</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="n">
+        <v>46037.37152777778</v>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>1</v>
+      </c>
+      <c r="F118" t="n">
+        <v>180</v>
+      </c>
+      <c r="G118" s="3" t="n">
+        <v>46045</v>
+      </c>
+      <c r="H118" t="n">
+        <v>9.49</v>
+      </c>
+      <c r="I118" t="n">
+        <v>188.3986</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>NVDA|180.0|2026-01-23|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>c424d059-5cb0-43ea-8326-c6d950c300e0</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="n">
+        <v>46035.59305555555</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>2</v>
+      </c>
+      <c r="F119" t="n">
+        <v>135</v>
+      </c>
+      <c r="G119" s="3" t="n">
+        <v>46038</v>
+      </c>
+      <c r="H119" t="n">
+        <v>4.87</v>
+      </c>
+      <c r="I119" t="n">
+        <v>139.6538</v>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>ABNB|135.0|2026-01-16|CALL|CLOSE</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="n">
+        <v>46035.59305555555</v>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>2</v>
+      </c>
+      <c r="F120" t="n">
+        <v>136</v>
+      </c>
+      <c r="G120" s="3" t="n">
+        <v>46045</v>
+      </c>
+      <c r="H120" t="n">
+        <v>4.81</v>
+      </c>
+      <c r="I120" t="n">
+        <v>139.6538</v>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>ABNB|136.0|2026-01-23|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="n">
+        <v>46036.36527777778</v>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>2</v>
+      </c>
+      <c r="F121" t="n">
+        <v>136</v>
+      </c>
+      <c r="G121" s="3" t="n">
+        <v>46045</v>
+      </c>
+      <c r="H121" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="I121" t="n">
+        <v>135.985</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>ABNB|136.0|2026-01-23|CALL|CLOSE</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="n">
+        <v>46036.36527777778</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>2</v>
+      </c>
+      <c r="F122" t="n">
+        <v>132</v>
+      </c>
+      <c r="G122" s="3" t="n">
+        <v>46045</v>
+      </c>
+      <c r="H122" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="I122" t="n">
+        <v>135.985</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>ABNB|132.0|2026-01-23|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="n">
+        <v>46036.49027777778</v>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>2</v>
+      </c>
+      <c r="F123" t="n">
+        <v>132</v>
+      </c>
+      <c r="G123" s="3" t="n">
+        <v>46045</v>
+      </c>
+      <c r="H123" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="I123" t="n">
+        <v>131.3668</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>ABNB|132.0|2026-01-23|CALL|CLOSE</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="n">
+        <v>46036.49027777778</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>2</v>
+      </c>
+      <c r="F124" t="n">
+        <v>129</v>
+      </c>
+      <c r="G124" s="3" t="n">
+        <v>46045</v>
+      </c>
+      <c r="H124" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="I124" t="n">
+        <v>131.3668</v>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>ABNB|129.0|2026-01-23|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixing income and dashboard
</commit_message>
<xml_diff>
--- a/cfm_journal/data/Juice_Ledger_Christie.xlsx
+++ b/cfm_journal/data/Juice_Ledger_Christie.xlsx
@@ -1,32 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-23148" yWindow="4188" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ledger" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="2">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,15 +23,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill/>
     </fill>
   </fills>
   <borders count="1">
@@ -56,18 +41,16 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -465,14 +448,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M124"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="20.42578125" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="19.28515625" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="32.7109375" customWidth="1" min="10" max="10"/>
-    <col width="33.28515625" customWidth="1" min="12" max="12"/>
-  </cols>
+  <dimension ref="A1:M143"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -7524,8 +7501,10 @@
           <t>Christie</t>
         </is>
       </c>
-      <c r="B108" s="1" t="n">
-        <v>46015.36180555556</v>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2025-12-24 8:41:00</t>
+        </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
@@ -7537,20 +7516,30 @@
           <t>NVDA</t>
         </is>
       </c>
-      <c r="E108" t="n">
-        <v>2</v>
-      </c>
-      <c r="F108" t="n">
-        <v>180</v>
-      </c>
-      <c r="G108" s="1" t="n">
-        <v>46024</v>
-      </c>
-      <c r="H108" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="I108" t="n">
-        <v>188.5525</v>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>2026-01-02 0:00:00</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>188.5525</t>
+        </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
@@ -7579,8 +7568,10 @@
           <t>Christie</t>
         </is>
       </c>
-      <c r="B109" s="1" t="n">
-        <v>46021.43194444444</v>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>2025-12-30 10:22:00</t>
+        </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
@@ -7592,20 +7583,30 @@
           <t>NVDA</t>
         </is>
       </c>
-      <c r="E109" t="n">
-        <v>2</v>
-      </c>
-      <c r="F109" t="n">
-        <v>180</v>
-      </c>
-      <c r="G109" s="1" t="n">
-        <v>46024</v>
-      </c>
-      <c r="H109" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="I109" t="n">
-        <v>188.4175</v>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>2026-01-02 0:00:00</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>8.8</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>188.4175</t>
+        </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
@@ -7634,8 +7635,10 @@
           <t>Christie</t>
         </is>
       </c>
-      <c r="B110" s="2" t="n">
-        <v>46029.38194444445</v>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>2026-01-07 9:10:00</t>
+        </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
@@ -7647,20 +7650,30 @@
           <t>NVDA</t>
         </is>
       </c>
-      <c r="E110" t="n">
-        <v>2</v>
-      </c>
-      <c r="F110" t="n">
-        <v>181</v>
-      </c>
-      <c r="G110" s="2" t="n">
-        <v>46038</v>
-      </c>
-      <c r="H110" t="n">
-        <v>11.3</v>
-      </c>
-      <c r="I110" t="n">
-        <v>190.6575</v>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>181</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>2026-01-16 0:00:00</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>190.6575</t>
+        </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
@@ -7689,8 +7702,10 @@
           <t>Christie</t>
         </is>
       </c>
-      <c r="B111" s="2" t="n">
-        <v>46036.39583333334</v>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>2026-01-14 9:30:00</t>
+        </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
@@ -7702,20 +7717,30 @@
           <t>NVDA</t>
         </is>
       </c>
-      <c r="E111" t="n">
-        <v>2</v>
-      </c>
-      <c r="F111" t="n">
-        <v>181</v>
-      </c>
-      <c r="G111" s="2" t="n">
-        <v>46038</v>
-      </c>
-      <c r="H111" t="n">
-        <v>2.77</v>
-      </c>
-      <c r="I111" t="n">
-        <v>181.7037</v>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>181</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>2026-01-16 0:00:00</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>2.77</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>181.7037</t>
+        </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
@@ -7744,8 +7769,10 @@
           <t>Christie</t>
         </is>
       </c>
-      <c r="B112" s="3" t="n">
-        <v>46036.39583333334</v>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2026-01-14 9:30:00</t>
+        </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
@@ -7757,20 +7784,30 @@
           <t>NVDA</t>
         </is>
       </c>
-      <c r="E112" t="n">
-        <v>1</v>
-      </c>
-      <c r="F112" t="n">
-        <v>181</v>
-      </c>
-      <c r="G112" s="3" t="n">
-        <v>46038</v>
-      </c>
-      <c r="H112" t="n">
-        <v>2.77</v>
-      </c>
-      <c r="I112" t="n">
-        <v>181.7037</v>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>181</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>2026-01-16 0:00:00</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>2.77</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>181.7037</t>
+        </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
@@ -7799,8 +7836,10 @@
           <t>Christie</t>
         </is>
       </c>
-      <c r="B113" s="3" t="n">
-        <v>46036.39583333334</v>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2026-01-14 9:30:00</t>
+        </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
@@ -7812,20 +7851,30 @@
           <t>NVDA</t>
         </is>
       </c>
-      <c r="E113" t="n">
-        <v>1</v>
-      </c>
-      <c r="F113" t="n">
-        <v>179</v>
-      </c>
-      <c r="G113" s="3" t="n">
-        <v>46038</v>
-      </c>
-      <c r="H113" t="n">
-        <v>4.06</v>
-      </c>
-      <c r="I113" t="n">
-        <v>181.7037</v>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>179</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>2026-01-16 0:00:00</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>4.06</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>181.7037</t>
+        </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
@@ -7854,8 +7903,10 @@
           <t>Christie</t>
         </is>
       </c>
-      <c r="B114" s="3" t="n">
-        <v>46036.39583333334</v>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2026-01-14 9:30:00</t>
+        </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
@@ -7867,20 +7918,30 @@
           <t>NVDA</t>
         </is>
       </c>
-      <c r="E114" t="n">
-        <v>2</v>
-      </c>
-      <c r="F114" t="n">
-        <v>179</v>
-      </c>
-      <c r="G114" s="3" t="n">
-        <v>46038</v>
-      </c>
-      <c r="H114" t="n">
-        <v>4.06</v>
-      </c>
-      <c r="I114" t="n">
-        <v>181.7037</v>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>179</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>2026-01-16 0:00:00</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>4.06</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>181.7037</t>
+        </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
@@ -7909,8 +7970,10 @@
           <t>Christie</t>
         </is>
       </c>
-      <c r="B115" s="3" t="n">
-        <v>46037.37152777778</v>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2026-01-15 8:55:00</t>
+        </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
@@ -7922,20 +7985,30 @@
           <t>NVDA</t>
         </is>
       </c>
-      <c r="E115" t="n">
-        <v>1</v>
-      </c>
-      <c r="F115" t="n">
-        <v>179</v>
-      </c>
-      <c r="G115" s="3" t="n">
-        <v>46038</v>
-      </c>
-      <c r="H115" t="n">
-        <v>9.59</v>
-      </c>
-      <c r="I115" t="n">
-        <v>188.3986</v>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>179</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>2026-01-16 0:00:00</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>9.59</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>188.3986</t>
+        </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
@@ -7964,8 +8037,10 @@
           <t>Christie</t>
         </is>
       </c>
-      <c r="B116" s="3" t="n">
-        <v>46037.37152777778</v>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2026-01-15 8:55:00</t>
+        </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
@@ -7977,20 +8052,30 @@
           <t>NVDA</t>
         </is>
       </c>
-      <c r="E116" t="n">
-        <v>2</v>
-      </c>
-      <c r="F116" t="n">
-        <v>179</v>
-      </c>
-      <c r="G116" s="3" t="n">
-        <v>46038</v>
-      </c>
-      <c r="H116" t="n">
-        <v>9.59</v>
-      </c>
-      <c r="I116" t="n">
-        <v>188.3986</v>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>179</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>2026-01-16 0:00:00</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>9.59</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>188.3986</t>
+        </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
@@ -8019,8 +8104,10 @@
           <t>Christie</t>
         </is>
       </c>
-      <c r="B117" s="3" t="n">
-        <v>46037.37152777778</v>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2026-01-15 8:55:00</t>
+        </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
@@ -8032,20 +8119,30 @@
           <t>NVDA</t>
         </is>
       </c>
-      <c r="E117" t="n">
-        <v>2</v>
-      </c>
-      <c r="F117" t="n">
-        <v>180</v>
-      </c>
-      <c r="G117" s="3" t="n">
-        <v>46045</v>
-      </c>
-      <c r="H117" t="n">
-        <v>9.49</v>
-      </c>
-      <c r="I117" t="n">
-        <v>188.3986</v>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>2026-01-23 0:00:00</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>9.49</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>188.3986</t>
+        </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
@@ -8074,8 +8171,10 @@
           <t>Christie</t>
         </is>
       </c>
-      <c r="B118" s="3" t="n">
-        <v>46037.37152777778</v>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2026-01-15 8:55:00</t>
+        </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
@@ -8087,20 +8186,30 @@
           <t>NVDA</t>
         </is>
       </c>
-      <c r="E118" t="n">
-        <v>1</v>
-      </c>
-      <c r="F118" t="n">
-        <v>180</v>
-      </c>
-      <c r="G118" s="3" t="n">
-        <v>46045</v>
-      </c>
-      <c r="H118" t="n">
-        <v>9.49</v>
-      </c>
-      <c r="I118" t="n">
-        <v>188.3986</v>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>2026-01-23 0:00:00</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>9.49</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>188.3986</t>
+        </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
@@ -8129,8 +8238,10 @@
           <t>Christie</t>
         </is>
       </c>
-      <c r="B119" s="3" t="n">
-        <v>46035.59305555555</v>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2026-01-13 14:14:00</t>
+        </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
@@ -8142,20 +8253,30 @@
           <t>ABNB</t>
         </is>
       </c>
-      <c r="E119" t="n">
-        <v>2</v>
-      </c>
-      <c r="F119" t="n">
-        <v>135</v>
-      </c>
-      <c r="G119" s="3" t="n">
-        <v>46038</v>
-      </c>
-      <c r="H119" t="n">
-        <v>4.87</v>
-      </c>
-      <c r="I119" t="n">
-        <v>139.6538</v>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>135</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>2026-01-16 0:00:00</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>4.87</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>139.6538</t>
+        </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
@@ -8184,8 +8305,10 @@
           <t>Christie</t>
         </is>
       </c>
-      <c r="B120" s="3" t="n">
-        <v>46035.59305555555</v>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2026-01-13 14:14:00</t>
+        </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
@@ -8197,20 +8320,30 @@
           <t>ABNB</t>
         </is>
       </c>
-      <c r="E120" t="n">
-        <v>2</v>
-      </c>
-      <c r="F120" t="n">
-        <v>136</v>
-      </c>
-      <c r="G120" s="3" t="n">
-        <v>46045</v>
-      </c>
-      <c r="H120" t="n">
-        <v>4.81</v>
-      </c>
-      <c r="I120" t="n">
-        <v>139.6538</v>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>2026-01-23 0:00:00</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>4.81</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>139.6538</t>
+        </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
@@ -8239,8 +8372,10 @@
           <t>Christie</t>
         </is>
       </c>
-      <c r="B121" s="3" t="n">
-        <v>46036.36527777778</v>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2026-01-14 8:46:00</t>
+        </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
@@ -8252,20 +8387,30 @@
           <t>ABNB</t>
         </is>
       </c>
-      <c r="E121" t="n">
-        <v>2</v>
-      </c>
-      <c r="F121" t="n">
-        <v>136</v>
-      </c>
-      <c r="G121" s="3" t="n">
-        <v>46045</v>
-      </c>
-      <c r="H121" t="n">
-        <v>3.63</v>
-      </c>
-      <c r="I121" t="n">
-        <v>135.985</v>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>2026-01-23 0:00:00</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>3.63</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>135.985</t>
+        </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
@@ -8294,8 +8439,10 @@
           <t>Christie</t>
         </is>
       </c>
-      <c r="B122" s="3" t="n">
-        <v>46036.36527777778</v>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-01-14 8:46:00</t>
+        </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
@@ -8307,20 +8454,30 @@
           <t>ABNB</t>
         </is>
       </c>
-      <c r="E122" t="n">
-        <v>2</v>
-      </c>
-      <c r="F122" t="n">
-        <v>132</v>
-      </c>
-      <c r="G122" s="3" t="n">
-        <v>46045</v>
-      </c>
-      <c r="H122" t="n">
-        <v>5.95</v>
-      </c>
-      <c r="I122" t="n">
-        <v>135.985</v>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>132</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>2026-01-23 0:00:00</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>5.95</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>135.985</t>
+        </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
@@ -8349,8 +8506,10 @@
           <t>Christie</t>
         </is>
       </c>
-      <c r="B123" s="3" t="n">
-        <v>46036.49027777778</v>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2026-01-14 11:46:00</t>
+        </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
@@ -8362,20 +8521,30 @@
           <t>ABNB</t>
         </is>
       </c>
-      <c r="E123" t="n">
-        <v>2</v>
-      </c>
-      <c r="F123" t="n">
-        <v>132</v>
-      </c>
-      <c r="G123" s="3" t="n">
-        <v>46045</v>
-      </c>
-      <c r="H123" t="n">
-        <v>2.28</v>
-      </c>
-      <c r="I123" t="n">
-        <v>131.3668</v>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>132</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>2026-01-23 0:00:00</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>2.28</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>131.3668</t>
+        </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
@@ -8404,8 +8573,10 @@
           <t>Christie</t>
         </is>
       </c>
-      <c r="B124" s="3" t="n">
-        <v>46036.49027777778</v>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2026-01-14 11:46:00</t>
+        </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
@@ -8417,39 +8588,1262 @@
           <t>ABNB</t>
         </is>
       </c>
-      <c r="E124" t="n">
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>2026-01-23 0:00:00</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>3.94</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>131.3668</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>ABNB|129.0|2026-01-23|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2026-01-22 8:31:00</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>2026-01-23 0:00:00</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>135.1325</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>ABNB|129.0|2026-01-23|CALL|CLOSE</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026-01-20 9:01:00</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>2026-01-23 0:00:00</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>179.8425</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>NVDA|180.0|2026-01-23|CALL|CLOSE</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>82f856ad-3a84-40d1-884d-02cc88c35c8a</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2026-01-20 9:01:00</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>2026-01-23 0:00:00</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>179.8425</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>NVDA|180.0|2026-01-23|CALL|CLOSE</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>c424d059-5cb0-43ea-8326-c6d950c300e0</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>2026-01-22 8:31:00</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>130</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>2026-01-30 0:00:00</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>5.85</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>135.1325</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>ABNB|130.0|2026-01-30|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>2026-01-26 9:04:00</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>130</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>2026-01-30 0:00:00</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>133.0513</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>ABNB|130.0|2026-01-30|CALL|CLOSE</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>2026-01-26 9:08:00</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>2026-02-06 0:00:00</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>5.52</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>133.1063</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>ABNB|129.0|2026-02-06|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2026-01-26 9:08:00</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>MARK</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>2026-02-06 0:00:00</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>5.52</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>133.1063</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>ABNB|129.0|2026-02-06|CALL|MARK</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>2cd0c5e468b54173be3aa830edbde00d</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2026-01-20 9:01:00</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>2026-01-23 0:00:00</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>6.6</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>179.8425</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>NVDA|175.0|2026-01-23|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>c424d059-5cb0-43ea-8326-c6d950c300e0</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>2026-01-22 8:32:00</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>2026-01-23 0:00:00</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>10.64</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>185.4167</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>NVDA|175.0|2026-01-23|CALL|CLOSE</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>c424d059-5cb0-43ea-8326-c6d950c300e0</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>2026-01-20 9:01:00</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>2026-01-23 0:00:00</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>6.6</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>179.8425</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>NVDA|175.0|2026-01-23|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>82f856ad-3a84-40d1-884d-02cc88c35c8a</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>2026-01-22 8:32:00</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>2026-01-23 0:00:00</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>10.64</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>185.4167</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>NVDA|175.0|2026-01-23|CALL|CLOSE</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>82f856ad-3a84-40d1-884d-02cc88c35c8a</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>2026-01-22 8:32:00</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>2026-01-30 0:00:00</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>11.79</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>185.4167</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>NVDA|175.0|2026-01-30|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>c424d059-5cb0-43ea-8326-c6d950c300e0</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B137" s="1" t="n">
+        <v>46050.36875</v>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>1</v>
+      </c>
+      <c r="F137" t="n">
+        <v>175</v>
+      </c>
+      <c r="G137" s="1" t="n">
+        <v>46052</v>
+      </c>
+      <c r="H137" t="n">
+        <v>17.02</v>
+      </c>
+      <c r="I137" t="n">
+        <v>191.6538</v>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>NVDA|175.0|2026-01-30|CALL|CLOSE</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>c424d059-5cb0-43ea-8326-c6d950c300e0</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>2026-01-22 8:32:00</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>2026-01-30 0:00:00</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>11.79</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>185.4167</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>NVDA|175.0|2026-01-30|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>82f856ad-3a84-40d1-884d-02cc88c35c8a</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>2026-01-28 8:51:00</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>CLOSE</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>2026-01-30 0:00:00</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>17.02</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>191.6538</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>NVDA|175.0|2026-01-30|CALL|CLOSE</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>82f856ad-3a84-40d1-884d-02cc88c35c8a</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B140" s="1" t="n">
+        <v>46050.36875</v>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
         <v>2</v>
       </c>
-      <c r="F124" t="n">
-        <v>129</v>
-      </c>
-      <c r="G124" s="3" t="n">
-        <v>46045</v>
-      </c>
-      <c r="H124" t="n">
-        <v>3.94</v>
-      </c>
-      <c r="I124" t="n">
-        <v>131.3668</v>
-      </c>
-      <c r="J124" t="inlineStr">
-        <is>
-          <t>ABNB|129.0|2026-01-23|CALL|OPEN</t>
-        </is>
-      </c>
-      <c r="K124" t="inlineStr">
-        <is>
-          <t>Call</t>
-        </is>
-      </c>
-      <c r="L124" t="inlineStr">
-        <is>
-          <t>2cd0c5e468b54173be3aa830edbde00d</t>
-        </is>
-      </c>
-      <c r="M124" t="inlineStr">
-        <is>
-          <t>cb86935f-1733-40f0-8ad6-fefb17700dd3</t>
+      <c r="F140" t="n">
+        <v>180</v>
+      </c>
+      <c r="G140" s="1" t="n">
+        <v>46059</v>
+      </c>
+      <c r="H140" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="I140" t="n">
+        <v>191.6538</v>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>NVDA|180.0|2026-02-06|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>82f856ad-3a84-40d1-884d-02cc88c35c8a</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B141" s="1" t="n">
+        <v>46050.36875</v>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>MARK</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>2</v>
+      </c>
+      <c r="F141" t="n">
+        <v>180</v>
+      </c>
+      <c r="G141" s="1" t="n">
+        <v>46059</v>
+      </c>
+      <c r="H141" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="I141" t="n">
+        <v>191.6538</v>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>NVDA|180.0|2026-02-06|CALL|MARK</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>82f856ad-3a84-40d1-884d-02cc88c35c8a</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B142" s="1" t="n">
+        <v>46050.36875</v>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>1</v>
+      </c>
+      <c r="F142" t="n">
+        <v>180</v>
+      </c>
+      <c r="G142" s="1" t="n">
+        <v>46059</v>
+      </c>
+      <c r="H142" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="I142" t="n">
+        <v>191.6538</v>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>NVDA|180.0|2026-02-06|CALL|OPEN</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>c424d059-5cb0-43ea-8326-c6d950c300e0</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="B143" s="1" t="n">
+        <v>46050.36875</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>MARK</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>1</v>
+      </c>
+      <c r="F143" t="n">
+        <v>180</v>
+      </c>
+      <c r="G143" s="1" t="n">
+        <v>46059</v>
+      </c>
+      <c r="H143" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="I143" t="n">
+        <v>191.6538</v>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>NVDA|180.0|2026-02-06|CALL|MARK</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>ffd625529d494de7a4481102e2be47fb</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>c424d059-5cb0-43ea-8326-c6d950c300e0</t>
         </is>
       </c>
     </row>

</xml_diff>